<commit_message>
Align API required fields with schema and add regression coverage.
</commit_message>
<xml_diff>
--- a/obspy/io/sitexml/tests/data/sera_site_no_owner.xlsx
+++ b/obspy/io/sitexml/tests/data/sera_site_no_owner.xlsx
@@ -1771,7 +1771,11 @@
           <t>0.43</t>
         </is>
       </c>
-      <c r="AI2" s="13" t="n"/>
+      <c r="AI2" s="13" t="inlineStr">
+        <is>
+          <t>Some title</t>
+        </is>
+      </c>
       <c r="AJ2" s="18" t="inlineStr">
         <is>
           <t>Author A.</t>

</xml_diff>